<commit_message>
Final commit before first presentation of MVP
</commit_message>
<xml_diff>
--- a/backend/carbon-credits/carbon-credits.xlsx
+++ b/backend/carbon-credits/carbon-credits.xlsx
@@ -15,10 +15,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.0"/>
-  </numFmts>
-  <fonts count="6">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,53 +27,22 @@
     <font>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1" tint="0.499984740745262"/>
-      <sz val="12"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
       <b val="1"/>
-      <color theme="1"/>
       <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color theme="1" tint="0.499984740745262"/>
-      <sz val="12"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <sz val="12"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="2" tint="-0.09997863704336681"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="6">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -84,50 +51,17 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
+      <left style="thin">
+        <color auto="1"/>
       </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="thin">
         <color auto="1"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
-      <bottom style="double">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="double">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
+      <bottom style="thin">
+        <color auto="1"/>
       </bottom>
       <diagonal/>
     </border>
@@ -141,52 +75,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="2" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -536,52 +430,52 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Units</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Inputs</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Baseline</t>
         </is>
       </c>
-      <c r="D1" s="15" t="n">
+      <c r="D1" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="E1" s="15" t="n">
+      <c r="E1" s="2" t="n">
         <v>2025</v>
       </c>
-      <c r="F1" s="15" t="n">
+      <c r="F1" s="2" t="n">
         <v>2026</v>
       </c>
-      <c r="G1" s="15" t="n">
+      <c r="G1" s="2" t="n">
         <v>2027</v>
       </c>
-      <c r="H1" s="15" t="n">
+      <c r="H1" s="2" t="n">
         <v>2028</v>
       </c>
-      <c r="I1" s="15" t="n">
+      <c r="I1" s="2" t="n">
         <v>2029</v>
       </c>
-      <c r="J1" s="15" t="n">
+      <c r="J1" s="2" t="n">
         <v>2030</v>
       </c>
-      <c r="K1" s="15" t="n">
+      <c r="K1" s="2" t="n">
         <v>2031</v>
       </c>
-      <c r="L1" s="15" t="n">
+      <c r="L1" s="2" t="n">
         <v>2032</v>
       </c>
-      <c r="M1" s="15" t="n">
+      <c r="M1" s="2" t="n">
         <v>2033</v>
       </c>
-      <c r="N1" s="15" t="n">
+      <c r="N1" s="2" t="n">
         <v>2034</v>
       </c>
     </row>

</xml_diff>